<commit_message>
V3.0 | 02.02.2024 -CICD- 02/02/2024 9:17:21 AM
</commit_message>
<xml_diff>
--- a/Carga Masiva/clientes.xlsx
+++ b/Carga Masiva/clientes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RepositoriosAEC\Acrux-Release\Carga Masiva\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20B80ECF-CADC-44AF-AFAB-0E4C49655BB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4760E150-5C76-4E93-91C6-854834E7E0AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21720" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="clientes" sheetId="1" r:id="rId1"/>
@@ -681,9 +681,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -721,7 +721,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -827,7 +827,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -969,7 +969,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -981,21 +981,21 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="11" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="15" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">

</xml_diff>